<commit_message>
feat: prioritize 4-star and 3-star hotels and cap 5-star to max 1-2 per location
</commit_message>
<xml_diff>
--- a/rate_sheets/Master_SriLanka_Hotel_Costing_Sheet.xlsx
+++ b/rate_sheets/Master_SriLanka_Hotel_Costing_Sheet.xlsx
@@ -1334,7 +1334,7 @@
         <v>Garden View Room</v>
       </c>
       <c r="F19" t="str">
-        <v>Winter Peak</v>
+        <v>Peak</v>
       </c>
       <c r="G19" t="str">
         <v>20 Dec 2026 - 10 Jan 2027</v>
@@ -1361,7 +1361,7 @@
         <v>0-1.99 years: FOC, 2-4.99 years: 30% of per-person rate, 5-9.99 years: 50% of per-person rate, 10-11.99 years: 70% of per-person rate, 12 years &amp; above: Counts as an Adult</v>
       </c>
       <c r="O19" t="str">
-        <v>NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB. Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked.</v>
+        <v>Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked. NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB.</v>
       </c>
       <c r="P19" t="str">
         <v>MBV 26-27  Foreign Rates from 01st May 2026 to 31st October 2027.pdf</v>
@@ -1384,7 +1384,7 @@
         <v>Garden View Room</v>
       </c>
       <c r="F20" t="str">
-        <v>Winter Peak</v>
+        <v>Peak</v>
       </c>
       <c r="G20" t="str">
         <v>20 Dec 2026 - 10 Jan 2027</v>
@@ -1411,7 +1411,7 @@
         <v>0-1.99 years: FOC, 2-4.99 years: 30% of per-person rate, 5-9.99 years: 50% of per-person rate, 10-11.99 years: 70% of per-person rate, 12 years &amp; above: Counts as an Adult</v>
       </c>
       <c r="O20" t="str">
-        <v>NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB. Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked.</v>
+        <v>Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked. NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB.</v>
       </c>
       <c r="P20" t="str">
         <v>MBV 26-27  Foreign Rates from 01st May 2026 to 31st October 2027.pdf</v>
@@ -1434,7 +1434,7 @@
         <v>Garden View Room</v>
       </c>
       <c r="F21" t="str">
-        <v>Winter Peak</v>
+        <v>Peak</v>
       </c>
       <c r="G21" t="str">
         <v>20 Dec 2026 - 10 Jan 2027</v>
@@ -1461,7 +1461,7 @@
         <v>0-1.99 years: FOC, 2-4.99 years: 30% of per-person rate, 5-9.99 years: 50% of per-person rate, 10-11.99 years: 70% of per-person rate, 12 years &amp; above: Counts as an Adult</v>
       </c>
       <c r="O21" t="str">
-        <v>NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB. Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked.</v>
+        <v>Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked. NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB.</v>
       </c>
       <c r="P21" t="str">
         <v>MBV 26-27  Foreign Rates from 01st May 2026 to 31st October 2027.pdf</v>
@@ -1484,7 +1484,7 @@
         <v>Sea View Room</v>
       </c>
       <c r="F22" t="str">
-        <v>Winter Peak</v>
+        <v>Peak</v>
       </c>
       <c r="G22" t="str">
         <v>20 Dec 2026 - 10 Jan 2027</v>
@@ -1511,7 +1511,7 @@
         <v>0-1.99 years: FOC, 2-4.99 years: 30% of per-person rate, 5-9.99 years: 50% of per-person rate, 10-11.99 years: 70% of per-person rate, 12 years &amp; above: Counts as an Adult</v>
       </c>
       <c r="O22" t="str">
-        <v>NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB. Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked.</v>
+        <v>Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked. NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB.</v>
       </c>
       <c r="P22" t="str">
         <v>MBV 26-27  Foreign Rates from 01st May 2026 to 31st October 2027.pdf</v>
@@ -1534,7 +1534,7 @@
         <v>Sea View Room</v>
       </c>
       <c r="F23" t="str">
-        <v>Winter Peak</v>
+        <v>Peak</v>
       </c>
       <c r="G23" t="str">
         <v>20 Dec 2026 - 10 Jan 2027</v>
@@ -1561,7 +1561,7 @@
         <v>0-1.99 years: FOC, 2-4.99 years: 30% of per-person rate, 5-9.99 years: 50% of per-person rate, 10-11.99 years: 70% of per-person rate, 12 years &amp; above: Counts as an Adult</v>
       </c>
       <c r="O23" t="str">
-        <v>NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB. Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked.</v>
+        <v>Cancellation within 45 days prior to arrival will be charged 100% of the room nights booked. NYE Supplement: USD 70 per person on HB, USD 80 per person on BB. Christmas Eve Supplement: USD 70 per person on HB, USD 85 per person on BB.</v>
       </c>
       <c r="P23" t="str">
         <v>MBV 26-27  Foreign Rates from 01st May 2026 to 31st October 2027.pdf</v>

</xml_diff>

<commit_message>
feat: migrate LLM fallback to gemini-2.5-flash, add PDF magic byte detection, and update costing master sheet
</commit_message>
<xml_diff>
--- a/rate_sheets/Master_SriLanka_Hotel_Costing_Sheet.xlsx
+++ b/rate_sheets/Master_SriLanka_Hotel_Costing_Sheet.xlsx
@@ -397,7 +397,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:P23"/>
+  <dimension ref="A1:P67"/>
   <cols>
     <col min="1" max="1" width="4.83203125" customWidth="1"/>
     <col min="2" max="2" width="16.83203125" customWidth="1"/>
@@ -1034,7 +1034,7 @@
         <v>Garden View Room</v>
       </c>
       <c r="F13" t="str">
-        <v>Winter</v>
+        <v>High</v>
       </c>
       <c r="G13" t="str">
         <v>01 November 2026 - 19 December 2026</v>
@@ -1084,7 +1084,7 @@
         <v>Garden View Room</v>
       </c>
       <c r="F14" t="str">
-        <v>Winter</v>
+        <v>High</v>
       </c>
       <c r="G14" t="str">
         <v>01 November 2026 - 19 December 2026</v>
@@ -1134,7 +1134,7 @@
         <v>Garden View Room</v>
       </c>
       <c r="F15" t="str">
-        <v>Winter</v>
+        <v>High</v>
       </c>
       <c r="G15" t="str">
         <v>01 November 2026 - 19 December 2026</v>
@@ -1184,7 +1184,7 @@
         <v>Sea View Room</v>
       </c>
       <c r="F16" t="str">
-        <v>Winter</v>
+        <v>High</v>
       </c>
       <c r="G16" t="str">
         <v>01 November 2026 - 19 December 2026</v>
@@ -1234,7 +1234,7 @@
         <v>Sea View Room</v>
       </c>
       <c r="F17" t="str">
-        <v>Winter</v>
+        <v>High</v>
       </c>
       <c r="G17" t="str">
         <v>01 November 2026 - 19 December 2026</v>
@@ -1284,7 +1284,7 @@
         <v>Sea View Room</v>
       </c>
       <c r="F18" t="str">
-        <v>Winter</v>
+        <v>High</v>
       </c>
       <c r="G18" t="str">
         <v>01 November 2026 - 19 December 2026</v>
@@ -1567,9 +1567,2209 @@
         <v>MBV 26-27  Foreign Rates from 01st May 2026 to 31st October 2027.pdf</v>
       </c>
     </row>
+    <row r="24">
+      <c r="A24">
+        <v>23</v>
+      </c>
+      <c r="B24" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C24" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D24" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E24" t="str">
+        <v>Poolview Single</v>
+      </c>
+      <c r="F24" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G24" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H24" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I24">
+        <v>50</v>
+      </c>
+      <c r="J24">
+        <v>60</v>
+      </c>
+      <c r="K24">
+        <v>75</v>
+      </c>
+      <c r="L24">
+        <v>90</v>
+      </c>
+      <c r="M24" t="str">
+        <v>-</v>
+      </c>
+      <c r="N24" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O24" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P24" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25">
+        <v>24</v>
+      </c>
+      <c r="B25" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C25" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D25" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E25" t="str">
+        <v>Poolview Double</v>
+      </c>
+      <c r="F25" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G25" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H25" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I25">
+        <v>60</v>
+      </c>
+      <c r="J25">
+        <v>80</v>
+      </c>
+      <c r="K25">
+        <v>110</v>
+      </c>
+      <c r="L25">
+        <v>120</v>
+      </c>
+      <c r="M25">
+        <v>20</v>
+      </c>
+      <c r="N25" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O25" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P25" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26">
+        <v>25</v>
+      </c>
+      <c r="B26" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C26" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D26" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E26" t="str">
+        <v>Poolview Triple</v>
+      </c>
+      <c r="F26" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G26" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H26" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I26">
+        <v>70</v>
+      </c>
+      <c r="J26">
+        <v>80</v>
+      </c>
+      <c r="K26">
+        <v>145</v>
+      </c>
+      <c r="L26">
+        <v>190</v>
+      </c>
+      <c r="M26">
+        <v>20</v>
+      </c>
+      <c r="N26" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O26" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P26" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27">
+        <v>26</v>
+      </c>
+      <c r="B27" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C27" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D27" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E27" t="str">
+        <v>Poolview Family</v>
+      </c>
+      <c r="F27" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G27" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H27" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I27">
+        <v>80</v>
+      </c>
+      <c r="J27">
+        <v>120</v>
+      </c>
+      <c r="K27">
+        <v>180</v>
+      </c>
+      <c r="L27">
+        <v>240</v>
+      </c>
+      <c r="M27">
+        <v>20</v>
+      </c>
+      <c r="N27" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O27" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P27" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28">
+        <v>27</v>
+      </c>
+      <c r="B28" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C28" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D28" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E28" t="str">
+        <v>Side Sea View - Deluxe Single</v>
+      </c>
+      <c r="F28" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G28" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H28" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I28">
+        <v>55</v>
+      </c>
+      <c r="J28">
+        <v>65</v>
+      </c>
+      <c r="K28">
+        <v>80</v>
+      </c>
+      <c r="L28">
+        <v>90</v>
+      </c>
+      <c r="M28" t="str">
+        <v>-</v>
+      </c>
+      <c r="N28" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O28" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P28" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29">
+        <v>28</v>
+      </c>
+      <c r="B29" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C29" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D29" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E29" t="str">
+        <v>Side Sea View - Deluxe Double</v>
+      </c>
+      <c r="F29" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G29" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H29" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I29">
+        <v>65</v>
+      </c>
+      <c r="J29">
+        <v>85</v>
+      </c>
+      <c r="K29">
+        <v>115</v>
+      </c>
+      <c r="L29">
+        <v>145</v>
+      </c>
+      <c r="M29">
+        <v>20</v>
+      </c>
+      <c r="N29" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O29" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P29" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30">
+        <v>29</v>
+      </c>
+      <c r="B30" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C30" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D30" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E30" t="str">
+        <v>Side Sea View - Deluxe Triple</v>
+      </c>
+      <c r="F30" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G30" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H30" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I30">
+        <v>75</v>
+      </c>
+      <c r="J30">
+        <v>105</v>
+      </c>
+      <c r="K30">
+        <v>150</v>
+      </c>
+      <c r="L30">
+        <v>195</v>
+      </c>
+      <c r="M30">
+        <v>20</v>
+      </c>
+      <c r="N30" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O30" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P30" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31">
+        <v>30</v>
+      </c>
+      <c r="B31" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C31" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D31" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E31" t="str">
+        <v>Side Sea View - Deluxe Family</v>
+      </c>
+      <c r="F31" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G31" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H31" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I31">
+        <v>85</v>
+      </c>
+      <c r="J31">
+        <v>125</v>
+      </c>
+      <c r="K31">
+        <v>185</v>
+      </c>
+      <c r="L31">
+        <v>245</v>
+      </c>
+      <c r="M31">
+        <v>20</v>
+      </c>
+      <c r="N31" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O31" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P31" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32">
+        <v>31</v>
+      </c>
+      <c r="B32" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C32" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D32" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E32" t="str">
+        <v>Direct Sea View - Deluxe Single</v>
+      </c>
+      <c r="F32" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G32" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H32" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I32">
+        <v>80</v>
+      </c>
+      <c r="J32">
+        <v>90</v>
+      </c>
+      <c r="K32">
+        <v>105</v>
+      </c>
+      <c r="L32">
+        <v>120</v>
+      </c>
+      <c r="M32" t="str">
+        <v>-</v>
+      </c>
+      <c r="N32" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O32" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P32" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33">
+        <v>32</v>
+      </c>
+      <c r="B33" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C33" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D33" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E33" t="str">
+        <v>Direct Sea View - Deluxe Double</v>
+      </c>
+      <c r="F33" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G33" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H33" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I33">
+        <v>90</v>
+      </c>
+      <c r="J33">
+        <v>110</v>
+      </c>
+      <c r="K33">
+        <v>140</v>
+      </c>
+      <c r="L33">
+        <v>170</v>
+      </c>
+      <c r="M33">
+        <v>20</v>
+      </c>
+      <c r="N33" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O33" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P33" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34">
+        <v>33</v>
+      </c>
+      <c r="B34" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C34" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D34" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E34" t="str">
+        <v>Direct Sea View - Deluxe Triple</v>
+      </c>
+      <c r="F34" t="str">
+        <v>Summer</v>
+      </c>
+      <c r="G34" t="str">
+        <v>01 May 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H34" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I34">
+        <v>100</v>
+      </c>
+      <c r="J34">
+        <v>130</v>
+      </c>
+      <c r="K34">
+        <v>170</v>
+      </c>
+      <c r="L34">
+        <v>220</v>
+      </c>
+      <c r="M34">
+        <v>20</v>
+      </c>
+      <c r="N34" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O34" t="str">
+        <v>All rates are in USD and non-commissionable. Rates are confidential and cannot be published on the internet. Check-in: 14:00hrs, Check-out: 12:00hrs. Individual bookings: payments 3 days prior to arrival. Group bookings (more than 5 rooms): 7 days prior to arrival. Any new taxes by the government will be borne by the Tour Operator/Travel Agent. Cancellation Policy: &gt;30 days prior to arrival - No charge; &lt;30 days prior to arrival - 50% charge; &lt;15 days prior to arrival - 100% charge; Cancellation during stay - 100% charge. Late check-out: Until 15:00hrs - 30% of one day room rate; Until 18:00hrs - 50% of one day room rate; After 18:00hrs - 100% of one day room rate.</v>
+      </c>
+      <c r="P34" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR SUMMER  2026.pdf</v>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35">
+        <v>34</v>
+      </c>
+      <c r="B35" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C35" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D35" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E35" t="str">
+        <v>Queen Rooms</v>
+      </c>
+      <c r="F35" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G35" t="str">
+        <v>01 Sep 2026 - 15 Oct 2026</v>
+      </c>
+      <c r="H35" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I35" t="str">
+        <v>-</v>
+      </c>
+      <c r="J35">
+        <v>110</v>
+      </c>
+      <c r="K35" t="str">
+        <v>-</v>
+      </c>
+      <c r="L35" t="str">
+        <v>-</v>
+      </c>
+      <c r="M35" t="str">
+        <v>-</v>
+      </c>
+      <c r="N35" t="str">
+        <v>-</v>
+      </c>
+      <c r="O35" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P35" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36">
+        <v>35</v>
+      </c>
+      <c r="B36" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C36" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D36" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E36" t="str">
+        <v>Queen Rooms</v>
+      </c>
+      <c r="F36" t="str">
+        <v>Mid</v>
+      </c>
+      <c r="G36" t="str">
+        <v>16 Oct 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H36" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I36" t="str">
+        <v>-</v>
+      </c>
+      <c r="J36">
+        <v>125</v>
+      </c>
+      <c r="K36" t="str">
+        <v>-</v>
+      </c>
+      <c r="L36" t="str">
+        <v>-</v>
+      </c>
+      <c r="M36" t="str">
+        <v>-</v>
+      </c>
+      <c r="N36" t="str">
+        <v>-</v>
+      </c>
+      <c r="O36" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P36" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37">
+        <v>36</v>
+      </c>
+      <c r="B37" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C37" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D37" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E37" t="str">
+        <v>Queen Rooms</v>
+      </c>
+      <c r="F37" t="str">
+        <v>High</v>
+      </c>
+      <c r="G37" t="str">
+        <v>01 Dec 2026 - 20 Dec 2026</v>
+      </c>
+      <c r="H37" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I37" t="str">
+        <v>-</v>
+      </c>
+      <c r="J37">
+        <v>140</v>
+      </c>
+      <c r="K37" t="str">
+        <v>-</v>
+      </c>
+      <c r="L37" t="str">
+        <v>-</v>
+      </c>
+      <c r="M37" t="str">
+        <v>-</v>
+      </c>
+      <c r="N37" t="str">
+        <v>-</v>
+      </c>
+      <c r="O37" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P37" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38">
+        <v>37</v>
+      </c>
+      <c r="B38" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C38" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D38" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E38" t="str">
+        <v>Queen Rooms</v>
+      </c>
+      <c r="F38" t="str">
+        <v>Peak</v>
+      </c>
+      <c r="G38" t="str">
+        <v>21 Dec 2026 - 10 Jan 2027</v>
+      </c>
+      <c r="H38" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I38" t="str">
+        <v>-</v>
+      </c>
+      <c r="J38">
+        <v>150</v>
+      </c>
+      <c r="K38" t="str">
+        <v>-</v>
+      </c>
+      <c r="L38" t="str">
+        <v>-</v>
+      </c>
+      <c r="M38" t="str">
+        <v>-</v>
+      </c>
+      <c r="N38" t="str">
+        <v>-</v>
+      </c>
+      <c r="O38" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P38" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39">
+        <v>38</v>
+      </c>
+      <c r="B39" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C39" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D39" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E39" t="str">
+        <v>Queen Rooms</v>
+      </c>
+      <c r="F39" t="str">
+        <v>High</v>
+      </c>
+      <c r="G39" t="str">
+        <v>11 Jan 2027 - 20 Mar 2027</v>
+      </c>
+      <c r="H39" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I39" t="str">
+        <v>-</v>
+      </c>
+      <c r="J39">
+        <v>140</v>
+      </c>
+      <c r="K39" t="str">
+        <v>-</v>
+      </c>
+      <c r="L39" t="str">
+        <v>-</v>
+      </c>
+      <c r="M39" t="str">
+        <v>-</v>
+      </c>
+      <c r="N39" t="str">
+        <v>-</v>
+      </c>
+      <c r="O39" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P39" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40">
+        <v>39</v>
+      </c>
+      <c r="B40" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C40" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D40" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E40" t="str">
+        <v>Queen Rooms</v>
+      </c>
+      <c r="F40" t="str">
+        <v>Mid</v>
+      </c>
+      <c r="G40" t="str">
+        <v>21 Mar 2027 - 04 Apr 2027</v>
+      </c>
+      <c r="H40" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I40" t="str">
+        <v>-</v>
+      </c>
+      <c r="J40">
+        <v>150</v>
+      </c>
+      <c r="K40" t="str">
+        <v>-</v>
+      </c>
+      <c r="L40" t="str">
+        <v>-</v>
+      </c>
+      <c r="M40" t="str">
+        <v>-</v>
+      </c>
+      <c r="N40" t="str">
+        <v>-</v>
+      </c>
+      <c r="O40" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P40" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41">
+        <v>40</v>
+      </c>
+      <c r="B41" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C41" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D41" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E41" t="str">
+        <v>Queen Rooms</v>
+      </c>
+      <c r="F41" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G41" t="str">
+        <v>05 Apr 2027 - 31 May 2027</v>
+      </c>
+      <c r="H41" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I41" t="str">
+        <v>-</v>
+      </c>
+      <c r="J41">
+        <v>110</v>
+      </c>
+      <c r="K41" t="str">
+        <v>-</v>
+      </c>
+      <c r="L41" t="str">
+        <v>-</v>
+      </c>
+      <c r="M41" t="str">
+        <v>-</v>
+      </c>
+      <c r="N41" t="str">
+        <v>-</v>
+      </c>
+      <c r="O41" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P41" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42">
+        <v>41</v>
+      </c>
+      <c r="B42" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C42" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D42" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E42" t="str">
+        <v>Prince Suits</v>
+      </c>
+      <c r="F42" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G42" t="str">
+        <v>01 Sep 2026 - 15 Oct 2026</v>
+      </c>
+      <c r="H42" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I42" t="str">
+        <v>-</v>
+      </c>
+      <c r="J42">
+        <v>150</v>
+      </c>
+      <c r="K42" t="str">
+        <v>-</v>
+      </c>
+      <c r="L42" t="str">
+        <v>-</v>
+      </c>
+      <c r="M42" t="str">
+        <v>-</v>
+      </c>
+      <c r="N42" t="str">
+        <v>-</v>
+      </c>
+      <c r="O42" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P42" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43">
+        <v>42</v>
+      </c>
+      <c r="B43" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C43" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D43" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E43" t="str">
+        <v>Prince Suits</v>
+      </c>
+      <c r="F43" t="str">
+        <v>Mid</v>
+      </c>
+      <c r="G43" t="str">
+        <v>16 Oct 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H43" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I43" t="str">
+        <v>-</v>
+      </c>
+      <c r="J43">
+        <v>175</v>
+      </c>
+      <c r="K43" t="str">
+        <v>-</v>
+      </c>
+      <c r="L43" t="str">
+        <v>-</v>
+      </c>
+      <c r="M43" t="str">
+        <v>-</v>
+      </c>
+      <c r="N43" t="str">
+        <v>-</v>
+      </c>
+      <c r="O43" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P43" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44">
+        <v>43</v>
+      </c>
+      <c r="B44" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C44" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D44" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E44" t="str">
+        <v>Prince Suits</v>
+      </c>
+      <c r="F44" t="str">
+        <v>High</v>
+      </c>
+      <c r="G44" t="str">
+        <v>01 Dec 2026 - 20 Dec 2026</v>
+      </c>
+      <c r="H44" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I44" t="str">
+        <v>-</v>
+      </c>
+      <c r="J44">
+        <v>200</v>
+      </c>
+      <c r="K44" t="str">
+        <v>-</v>
+      </c>
+      <c r="L44" t="str">
+        <v>-</v>
+      </c>
+      <c r="M44" t="str">
+        <v>-</v>
+      </c>
+      <c r="N44" t="str">
+        <v>-</v>
+      </c>
+      <c r="O44" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P44" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45">
+        <v>44</v>
+      </c>
+      <c r="B45" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C45" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D45" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E45" t="str">
+        <v>Prince Suits</v>
+      </c>
+      <c r="F45" t="str">
+        <v>Peak</v>
+      </c>
+      <c r="G45" t="str">
+        <v>21 Dec 2026 - 10 Jan 2027</v>
+      </c>
+      <c r="H45" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I45" t="str">
+        <v>-</v>
+      </c>
+      <c r="J45">
+        <v>250</v>
+      </c>
+      <c r="K45" t="str">
+        <v>-</v>
+      </c>
+      <c r="L45" t="str">
+        <v>-</v>
+      </c>
+      <c r="M45" t="str">
+        <v>-</v>
+      </c>
+      <c r="N45" t="str">
+        <v>-</v>
+      </c>
+      <c r="O45" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P45" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46">
+        <v>45</v>
+      </c>
+      <c r="B46" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C46" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D46" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E46" t="str">
+        <v>Prince Suits</v>
+      </c>
+      <c r="F46" t="str">
+        <v>High</v>
+      </c>
+      <c r="G46" t="str">
+        <v>11 Jan 2027 - 20 Mar 2027</v>
+      </c>
+      <c r="H46" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I46" t="str">
+        <v>-</v>
+      </c>
+      <c r="J46">
+        <v>200</v>
+      </c>
+      <c r="K46" t="str">
+        <v>-</v>
+      </c>
+      <c r="L46" t="str">
+        <v>-</v>
+      </c>
+      <c r="M46" t="str">
+        <v>-</v>
+      </c>
+      <c r="N46" t="str">
+        <v>-</v>
+      </c>
+      <c r="O46" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P46" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47">
+        <v>46</v>
+      </c>
+      <c r="B47" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C47" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D47" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E47" t="str">
+        <v>Prince Suits</v>
+      </c>
+      <c r="F47" t="str">
+        <v>Mid</v>
+      </c>
+      <c r="G47" t="str">
+        <v>21 Mar 2027 - 04 Apr 2027</v>
+      </c>
+      <c r="H47" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I47" t="str">
+        <v>-</v>
+      </c>
+      <c r="J47">
+        <v>250</v>
+      </c>
+      <c r="K47" t="str">
+        <v>-</v>
+      </c>
+      <c r="L47" t="str">
+        <v>-</v>
+      </c>
+      <c r="M47" t="str">
+        <v>-</v>
+      </c>
+      <c r="N47" t="str">
+        <v>-</v>
+      </c>
+      <c r="O47" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P47" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48">
+        <v>47</v>
+      </c>
+      <c r="B48" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C48" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D48" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E48" t="str">
+        <v>Prince Suits</v>
+      </c>
+      <c r="F48" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G48" t="str">
+        <v>05 Apr 2027 - 31 May 2027</v>
+      </c>
+      <c r="H48" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I48" t="str">
+        <v>-</v>
+      </c>
+      <c r="J48">
+        <v>150</v>
+      </c>
+      <c r="K48" t="str">
+        <v>-</v>
+      </c>
+      <c r="L48" t="str">
+        <v>-</v>
+      </c>
+      <c r="M48" t="str">
+        <v>-</v>
+      </c>
+      <c r="N48" t="str">
+        <v>-</v>
+      </c>
+      <c r="O48" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P48" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49">
+        <v>48</v>
+      </c>
+      <c r="B49" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C49" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D49" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E49" t="str">
+        <v>Kings Residence</v>
+      </c>
+      <c r="F49" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G49" t="str">
+        <v>01 Sep 2026 - 15 Oct 2026</v>
+      </c>
+      <c r="H49" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I49" t="str">
+        <v>-</v>
+      </c>
+      <c r="J49">
+        <v>200</v>
+      </c>
+      <c r="K49" t="str">
+        <v>-</v>
+      </c>
+      <c r="L49" t="str">
+        <v>-</v>
+      </c>
+      <c r="M49" t="str">
+        <v>-</v>
+      </c>
+      <c r="N49" t="str">
+        <v>-</v>
+      </c>
+      <c r="O49" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P49" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50">
+        <v>49</v>
+      </c>
+      <c r="B50" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C50" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D50" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E50" t="str">
+        <v>Kings Residence</v>
+      </c>
+      <c r="F50" t="str">
+        <v>Mid</v>
+      </c>
+      <c r="G50" t="str">
+        <v>16 Oct 2026 - 30 Nov 2026</v>
+      </c>
+      <c r="H50" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I50" t="str">
+        <v>-</v>
+      </c>
+      <c r="J50">
+        <v>250</v>
+      </c>
+      <c r="K50" t="str">
+        <v>-</v>
+      </c>
+      <c r="L50" t="str">
+        <v>-</v>
+      </c>
+      <c r="M50" t="str">
+        <v>-</v>
+      </c>
+      <c r="N50" t="str">
+        <v>-</v>
+      </c>
+      <c r="O50" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P50" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="51">
+      <c r="A51">
+        <v>50</v>
+      </c>
+      <c r="B51" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C51" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D51" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E51" t="str">
+        <v>Kings Residence</v>
+      </c>
+      <c r="F51" t="str">
+        <v>High</v>
+      </c>
+      <c r="G51" t="str">
+        <v>01 Dec 2026 - 20 Dec 2026</v>
+      </c>
+      <c r="H51" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I51" t="str">
+        <v>-</v>
+      </c>
+      <c r="J51">
+        <v>300</v>
+      </c>
+      <c r="K51" t="str">
+        <v>-</v>
+      </c>
+      <c r="L51" t="str">
+        <v>-</v>
+      </c>
+      <c r="M51" t="str">
+        <v>-</v>
+      </c>
+      <c r="N51" t="str">
+        <v>-</v>
+      </c>
+      <c r="O51" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P51" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52">
+        <v>51</v>
+      </c>
+      <c r="B52" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C52" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D52" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E52" t="str">
+        <v>Kings Residence</v>
+      </c>
+      <c r="F52" t="str">
+        <v>Peak</v>
+      </c>
+      <c r="G52" t="str">
+        <v>21 Dec 2026 - 10 Jan 2027</v>
+      </c>
+      <c r="H52" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I52" t="str">
+        <v>-</v>
+      </c>
+      <c r="J52">
+        <v>350</v>
+      </c>
+      <c r="K52" t="str">
+        <v>-</v>
+      </c>
+      <c r="L52" t="str">
+        <v>-</v>
+      </c>
+      <c r="M52" t="str">
+        <v>-</v>
+      </c>
+      <c r="N52" t="str">
+        <v>-</v>
+      </c>
+      <c r="O52" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P52" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53">
+        <v>52</v>
+      </c>
+      <c r="B53" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C53" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D53" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E53" t="str">
+        <v>Kings Residence</v>
+      </c>
+      <c r="F53" t="str">
+        <v>High</v>
+      </c>
+      <c r="G53" t="str">
+        <v>11 Jan 2027 - 20 Mar 2027</v>
+      </c>
+      <c r="H53" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I53" t="str">
+        <v>-</v>
+      </c>
+      <c r="J53">
+        <v>300</v>
+      </c>
+      <c r="K53" t="str">
+        <v>-</v>
+      </c>
+      <c r="L53" t="str">
+        <v>-</v>
+      </c>
+      <c r="M53" t="str">
+        <v>-</v>
+      </c>
+      <c r="N53" t="str">
+        <v>-</v>
+      </c>
+      <c r="O53" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P53" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54">
+        <v>53</v>
+      </c>
+      <c r="B54" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C54" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D54" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E54" t="str">
+        <v>Kings Residence</v>
+      </c>
+      <c r="F54" t="str">
+        <v>Mid</v>
+      </c>
+      <c r="G54" t="str">
+        <v>21 Mar 2027 - 04 Apr 2027</v>
+      </c>
+      <c r="H54" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I54" t="str">
+        <v>-</v>
+      </c>
+      <c r="J54">
+        <v>350</v>
+      </c>
+      <c r="K54" t="str">
+        <v>-</v>
+      </c>
+      <c r="L54" t="str">
+        <v>-</v>
+      </c>
+      <c r="M54" t="str">
+        <v>-</v>
+      </c>
+      <c r="N54" t="str">
+        <v>-</v>
+      </c>
+      <c r="O54" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P54" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="55">
+      <c r="A55">
+        <v>54</v>
+      </c>
+      <c r="B55" t="str">
+        <v>Sri Lanka</v>
+      </c>
+      <c r="C55" t="str">
+        <v>3-star</v>
+      </c>
+      <c r="D55" t="str">
+        <v>Amila Vidanapathirana</v>
+      </c>
+      <c r="E55" t="str">
+        <v>Kings Residence</v>
+      </c>
+      <c r="F55" t="str">
+        <v>Low</v>
+      </c>
+      <c r="G55" t="str">
+        <v>05 Apr 2027 - 31 May 2027</v>
+      </c>
+      <c r="H55" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I55" t="str">
+        <v>-</v>
+      </c>
+      <c r="J55">
+        <v>200</v>
+      </c>
+      <c r="K55" t="str">
+        <v>-</v>
+      </c>
+      <c r="L55" t="str">
+        <v>-</v>
+      </c>
+      <c r="M55" t="str">
+        <v>-</v>
+      </c>
+      <c r="N55" t="str">
+        <v>-</v>
+      </c>
+      <c r="O55" t="str">
+        <v>Rates are exclusive of applicable taxes. 50% non-refundable deposit required for reservation confirmation. Rates are subject to change based on market conditions, special events, seasonal periods, and operational factors. Valid until 31 May 2027.</v>
+      </c>
+      <c r="P55" t="str">
+        <v>Travel Agent Rate Sheet - Prince of Galle.pdf</v>
+      </c>
+    </row>
+    <row r="56">
+      <c r="A56">
+        <v>55</v>
+      </c>
+      <c r="B56" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C56" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D56" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E56" t="str">
+        <v>POOLVIEW - Single</v>
+      </c>
+      <c r="F56" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G56" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H56" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I56">
+        <v>95</v>
+      </c>
+      <c r="J56">
+        <v>105</v>
+      </c>
+      <c r="K56">
+        <v>120</v>
+      </c>
+      <c r="L56">
+        <v>135</v>
+      </c>
+      <c r="M56" t="str">
+        <v>-</v>
+      </c>
+      <c r="N56" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O56" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P56" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="57">
+      <c r="A57">
+        <v>56</v>
+      </c>
+      <c r="B57" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C57" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D57" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E57" t="str">
+        <v>POOLVIEW - Double</v>
+      </c>
+      <c r="F57" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G57" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H57" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I57">
+        <v>105</v>
+      </c>
+      <c r="J57">
+        <v>125</v>
+      </c>
+      <c r="K57">
+        <v>155</v>
+      </c>
+      <c r="L57">
+        <v>185</v>
+      </c>
+      <c r="M57">
+        <v>20</v>
+      </c>
+      <c r="N57" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O57" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P57" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58">
+        <v>57</v>
+      </c>
+      <c r="B58" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C58" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D58" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E58" t="str">
+        <v>POOLVIEW - Tripple</v>
+      </c>
+      <c r="F58" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G58" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H58" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I58">
+        <v>115</v>
+      </c>
+      <c r="J58">
+        <v>145</v>
+      </c>
+      <c r="K58">
+        <v>190</v>
+      </c>
+      <c r="L58">
+        <v>235</v>
+      </c>
+      <c r="M58">
+        <v>20</v>
+      </c>
+      <c r="N58" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O58" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P58" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59">
+        <v>58</v>
+      </c>
+      <c r="B59" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C59" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D59" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E59" t="str">
+        <v>POOLVIEW - Family</v>
+      </c>
+      <c r="F59" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G59" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H59" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I59">
+        <v>125</v>
+      </c>
+      <c r="J59">
+        <v>165</v>
+      </c>
+      <c r="K59">
+        <v>225</v>
+      </c>
+      <c r="L59">
+        <v>285</v>
+      </c>
+      <c r="M59">
+        <v>20</v>
+      </c>
+      <c r="N59" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O59" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P59" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60">
+        <v>59</v>
+      </c>
+      <c r="B60" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C60" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D60" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E60" t="str">
+        <v>SIDE SEA VIEW - DELUXE - Single</v>
+      </c>
+      <c r="F60" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G60" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H60" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I60">
+        <v>100</v>
+      </c>
+      <c r="J60">
+        <v>110</v>
+      </c>
+      <c r="K60">
+        <v>125</v>
+      </c>
+      <c r="L60">
+        <v>140</v>
+      </c>
+      <c r="M60" t="str">
+        <v>-</v>
+      </c>
+      <c r="N60" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O60" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P60" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61">
+        <v>60</v>
+      </c>
+      <c r="B61" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C61" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D61" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E61" t="str">
+        <v>SIDE SEA VIEW - DELUXE - Double</v>
+      </c>
+      <c r="F61" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G61" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H61" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I61">
+        <v>110</v>
+      </c>
+      <c r="J61">
+        <v>130</v>
+      </c>
+      <c r="K61">
+        <v>160</v>
+      </c>
+      <c r="L61">
+        <v>190</v>
+      </c>
+      <c r="M61">
+        <v>20</v>
+      </c>
+      <c r="N61" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O61" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P61" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="62">
+      <c r="A62">
+        <v>61</v>
+      </c>
+      <c r="B62" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C62" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D62" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E62" t="str">
+        <v>SIDE SEA VIEW - DELUXE - Tripple</v>
+      </c>
+      <c r="F62" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G62" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H62" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I62">
+        <v>120</v>
+      </c>
+      <c r="J62">
+        <v>150</v>
+      </c>
+      <c r="K62">
+        <v>195</v>
+      </c>
+      <c r="L62">
+        <v>240</v>
+      </c>
+      <c r="M62">
+        <v>20</v>
+      </c>
+      <c r="N62" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O62" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P62" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="63">
+      <c r="A63">
+        <v>62</v>
+      </c>
+      <c r="B63" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C63" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D63" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E63" t="str">
+        <v>SIDE SEA VIEW - DELUXE - Family</v>
+      </c>
+      <c r="F63" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G63" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H63" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I63">
+        <v>130</v>
+      </c>
+      <c r="J63">
+        <v>170</v>
+      </c>
+      <c r="K63">
+        <v>230</v>
+      </c>
+      <c r="L63">
+        <v>290</v>
+      </c>
+      <c r="M63">
+        <v>20</v>
+      </c>
+      <c r="N63" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O63" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P63" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64">
+        <v>63</v>
+      </c>
+      <c r="B64" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C64" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D64" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E64" t="str">
+        <v>DIRECT SEA VIEW - DELUXE - Single</v>
+      </c>
+      <c r="F64" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G64" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H64" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I64">
+        <v>125</v>
+      </c>
+      <c r="J64">
+        <v>135</v>
+      </c>
+      <c r="K64">
+        <v>150</v>
+      </c>
+      <c r="L64">
+        <v>165</v>
+      </c>
+      <c r="M64" t="str">
+        <v>-</v>
+      </c>
+      <c r="N64" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O64" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P64" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="65">
+      <c r="A65">
+        <v>64</v>
+      </c>
+      <c r="B65" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C65" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D65" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E65" t="str">
+        <v>DIRECT SEA VIEW - DELUXE - Double</v>
+      </c>
+      <c r="F65" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G65" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H65" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I65">
+        <v>135</v>
+      </c>
+      <c r="J65">
+        <v>155</v>
+      </c>
+      <c r="K65">
+        <v>185</v>
+      </c>
+      <c r="L65">
+        <v>215</v>
+      </c>
+      <c r="M65">
+        <v>20</v>
+      </c>
+      <c r="N65" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O65" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P65" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66">
+        <v>65</v>
+      </c>
+      <c r="B66" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C66" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D66" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E66" t="str">
+        <v>DIRECT SEA VIEW - DELUXE - Tripple</v>
+      </c>
+      <c r="F66" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G66" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H66" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I66">
+        <v>145</v>
+      </c>
+      <c r="J66">
+        <v>175</v>
+      </c>
+      <c r="K66">
+        <v>220</v>
+      </c>
+      <c r="L66">
+        <v>265</v>
+      </c>
+      <c r="M66">
+        <v>20</v>
+      </c>
+      <c r="N66" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O66" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P66" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67">
+        <v>66</v>
+      </c>
+      <c r="B67" t="str">
+        <v>Mirissa</v>
+      </c>
+      <c r="C67" t="str">
+        <v>4-star</v>
+      </c>
+      <c r="D67" t="str">
+        <v>Randiya Sea View Hotel</v>
+      </c>
+      <c r="E67" t="str">
+        <v>DIRECT SEA VIEW - DELUXE - Family</v>
+      </c>
+      <c r="F67" t="str">
+        <v>Winter</v>
+      </c>
+      <c r="G67" t="str">
+        <v>01 Dec 2026 - 30 Apr 2027</v>
+      </c>
+      <c r="H67" t="str">
+        <v>USD</v>
+      </c>
+      <c r="I67">
+        <v>155</v>
+      </c>
+      <c r="J67">
+        <v>195</v>
+      </c>
+      <c r="K67">
+        <v>255</v>
+      </c>
+      <c r="L67">
+        <v>315</v>
+      </c>
+      <c r="M67">
+        <v>20</v>
+      </c>
+      <c r="N67" t="str">
+        <v>Child Supplement - 8 USD (5 to 12 years on BB Basis), 18 USD (5 to 12 years on HB Basis), 25 USD (5 to 12 years on FB Basis)</v>
+      </c>
+      <c r="O67" t="str">
+        <v>Cancellation: &gt;30 days no charge, &lt;30 days 50%, &lt;15 days 100%. Check-in 14:00, Check-out 12:00. Late check-out charges apply.</v>
+      </c>
+      <c r="P67" t="str">
+        <v>SPECIAL TRAVEL AGENT RATE FOR WINTER 2026 - 2027 01ST DECEMBR  2026 – 30th APRIL</v>
+      </c>
+    </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:P23"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:P67"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>